<commit_message>
reorganisation, add windows environment compatibility
</commit_message>
<xml_diff>
--- a/Poll normaliser.xlsx
+++ b/Poll normaliser.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djhir\source\repos\Polling Analyser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C490F73D-06FC-4150-A395-1597B9987468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719EBDA9-E95D-4BA1-BA57-A9343E1C0759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="435" yWindow="885" windowWidth="29610" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
+    <workbookView xWindow="945" yWindow="6300" windowWidth="29610" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -471,16 +471,16 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B2">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E2" t="e">
         <v>#N/A</v>
@@ -495,29 +495,29 @@
         <v>#N/A</v>
       </c>
       <c r="I2">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="K2">
         <f>SUMIF(A2:I2,"&gt;0")</f>
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:I4" si="0">A2*100/$K$2</f>
-        <v>23.762376237623762</v>
+        <v>23.404255319148938</v>
       </c>
       <c r="B4">
         <f t="shared" si="0"/>
-        <v>27.722772277227723</v>
+        <v>30.851063829787233</v>
       </c>
       <c r="C4">
         <f t="shared" si="0"/>
-        <v>13.861386138613861</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>22.772277227722771</v>
+        <v>26.595744680851062</v>
       </c>
       <c r="E4" t="e">
         <f t="shared" si="0"/>
@@ -537,7 +537,7 @@
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>11.881188118811881</v>
+        <v>6.3829787234042552</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -548,19 +548,19 @@
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f>_xlfn.IFNA(A4,0)</f>
-        <v>23.762376237623762</v>
+        <v>23.404255319148938</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" ref="B6:I6" si="1">_xlfn.IFNA(B4,0)</f>
-        <v>27.722772277227723</v>
+        <v>30.851063829787233</v>
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>13.861386138613861</v>
+        <v>12.76595744680851</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="1"/>
-        <v>22.772277227722771</v>
+        <v>26.595744680851062</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="1"/>
@@ -580,7 +580,7 @@
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>11.881188118811881</v>
+        <v>6.3829787234042552</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -619,7 +619,7 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K8">
         <f>SUMPRODUCT(A6:I6,A7:I7)</f>
-        <v>52.22930693069307</v>
+        <v>52.37</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
2022fed live simulated changes
-includes adjustment to regional variability that affect non-live federal elections
</commit_message>
<xml_diff>
--- a/Poll normaliser.xlsx
+++ b/Poll normaliser.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djhir\source\repos\Polling Analyser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{108343B9-2184-48F6-8462-3C0B22C87AD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67668E50-9124-4A56-B49B-8FA3DBE53EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3975" yWindow="9795" windowWidth="29610" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
+    <workbookView xWindow="7200" yWindow="2730" windowWidth="29610" windowHeight="16350" xr2:uid="{6D0FA6D2-DD42-4A2B-A7FB-8B25D0B69908}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -471,16 +471,16 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B2">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C2">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D2">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E2" t="e">
         <v>#N/A</v>
@@ -495,7 +495,7 @@
         <v>#N/A</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K2">
         <f>SUMIF(A2:I2,"&gt;0")</f>
@@ -505,19 +505,19 @@
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" ref="A4:I4" si="0">A2*100/$K$2</f>
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B4">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D4">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E4" t="e">
         <f t="shared" si="0"/>
@@ -537,7 +537,7 @@
       </c>
       <c r="I4">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -548,19 +548,19 @@
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <f>_xlfn.IFNA(A4,0)</f>
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B6" s="1">
         <f t="shared" ref="B6:I6" si="1">_xlfn.IFNA(B4,0)</f>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C6" s="1">
         <f t="shared" si="1"/>
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D6" s="1">
         <f t="shared" si="1"/>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="1"/>
@@ -580,7 +580,7 @@
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -619,7 +619,7 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="K8">
         <f>SUMPRODUCT(A6:I6,A7:I7)</f>
-        <v>48.272100000000002</v>
+        <v>51.7166</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>